<commit_message>
Freeze pass: consistency fixes across the paper, summary, model, appendix and pages
- Paper 39.1 re-exported (17 October): equations restored, 52 pages, authorship note on page 36; cross-check, PCA, GOES range, Table A2 growth basis, moat lead times, Operator X wording, Section II wording, charts and FRED reference made consistent
- Four-page summary aligned with the paper (bands, timing, Operator H, claims limited to what was reviewed)
- Valuation model: sheet references quoted for Excel, cover and Section II note updated, author set; same values
- Appendix B: numbers stored as numbers, correct PC1 loadings, GOES range and lead-time level note
- Pages: AI statement rewritten around concrete judgment calls; correction log extended; annex unposted; hide-sources fixed; dates 17 October

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TVKuA7cByrMM7fRzvfpzTB
</commit_message>
<xml_diff>
--- a/research/files/SPG-Appendix-B-Data-and-Reproducibility-v39.xlsx
+++ b/research/files/SPG-Appendix-B-Data-and-Reproducibility-v39.xlsx
@@ -16,7 +16,7 @@
     <sheet name="GOES Bridge" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Constraint Data'!$A$1:$F$33</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Constraint Data'!$A$1:$F$34</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Constraint Data'!$1:$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Correlation!$A$1:$G$13</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Correlation!$1:$1</definedName>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="100">
   <si>
     <t xml:space="preserve">SIMANCAS CAPITAL  |  LORENZO FRASCOLLA</t>
   </si>
@@ -91,13 +91,13 @@
     <t xml:space="preserve">Result 4</t>
   </si>
   <si>
-    <t xml:space="preserve">AI data-center transformers absorb ~35-40% of the annual GROWTH in GOES demand (range ~20-50% across reasonable inputs), not 42% of total or of installed supply. The claim is reframed accordingly.</t>
+    <t xml:space="preserve">AI data-center transformers absorb ~35-40% of the annual GROWTH in GOES demand (central case ~36%; range ~20-55% across the sensitivity grid on the GOES Bridge tab), not 42% of total or of installed supply. The claim is reframed accordingly.</t>
   </si>
   <si>
     <t xml:space="preserve">Caveats</t>
   </si>
   <si>
-    <t xml:space="preserve">Annual anchors are interpolated/estimated where only range data exist; the GOES and labor series are tightness proxies, not audited price indices. Treat the exact coefficients as defensible magnitudes, not precise measurements. Sources are listed on each tab.</t>
+    <t xml:space="preserve">Annual anchors are interpolated/estimated where only range data exist; the GOES and labor series are tightness proxies, not audited price indices. Treat the exact coefficients as defensible magnitudes, not precise measurements. Sources are listed on each tab. The transformer lead-time series (21 months in 2018 to 53 months in 2025) is a tightness proxy built from large-power-transformer industry ranges. Its level runs above the paper's own lead-time figures (Table A2: 38 weeks in 2018 Q1 to 210 weeks in 2026 Q1; text: 128 to 144 weeks on average by 2026). Only year-over-year changes enter the correlation and principal-component results, so the level difference does not drive them.</t>
   </si>
   <si>
     <t xml:space="preserve">CONTENTS</t>
@@ -136,28 +136,8 @@
     <t xml:space="preserve">Lorenzo Frascolla  |  Simancas Capital</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Constraint Data
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Five constraint series, 2018-2025, in levels and as year-over-year changes, with sources.</t>
-    </r>
+    <t xml:space="preserve">Constraint Data
+Five constraint series, 2018-2025, in levels and as year-over-year changes, with sources.</t>
   </si>
   <si>
     <t xml:space="preserve">Contents</t>
@@ -181,30 +161,6 @@
     <t xml:space="preserve">HV labor idx</t>
   </si>
   <si>
-    <t xml:space="preserve">2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025</t>
-  </si>
-  <si>
     <t xml:space="preserve">Year-over-year changes (used for correlation)</t>
   </si>
   <si>
@@ -226,28 +182,11 @@
     <t xml:space="preserve">HV labor idx: proxy for high-voltage winding skilled-labor tightness (rising). Author estimate from trade/OEM commentary.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Correlation
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Pairwise correlations of year-over-year changes (live CORREL formulas).</t>
-    </r>
+    <t xml:space="preserve">Note: the transformer series is a tightness proxy; its level runs above the paper's Table A2 lead times. Only the year-over-year changes above enter the correlations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation
+Pairwise correlations of year-over-year changes (live CORREL formulas).</t>
   </si>
   <si>
     <t xml:space="preserve">Interconnect</t>
@@ -271,28 +210,8 @@
     <t xml:space="preserve">NEPA is negatively correlated with the supply constraints (it improved over the period); interconnection is weakly linked.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Principal Components
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Share of variance explained by the first principal component of the change-correlation matrix.</t>
-    </r>
+    <t xml:space="preserve">Principal Components
+Share of variance explained by the first principal component of the change-correlation matrix.</t>
   </si>
   <si>
     <t xml:space="preserve">Computed in Python (numpy.linalg.eigh) on the Correlation tab matrix; recompute if data change.</t>
@@ -310,55 +229,26 @@
     <t xml:space="preserve">All five constraints</t>
   </si>
   <si>
-    <t xml:space="preserve">49.6%</t>
-  </si>
-  <si>
     <t xml:space="preserve">one common factor, NEPA loads inversely</t>
   </si>
   <si>
     <t xml:space="preserve">Four supply-side (ex-NEPA)</t>
   </si>
   <si>
-    <t xml:space="preserve">61.9%</t>
-  </si>
-  <si>
     <t xml:space="preserve">interconnection loads weakly</t>
   </si>
   <si>
     <t xml:space="preserve">Manufacturing cluster (3)</t>
   </si>
   <si>
-    <t xml:space="preserve">80.0%</t>
-  </si>
-  <si>
     <t xml:space="preserve">transformer/GOES/labor as one factor</t>
   </si>
   <si>
-    <t xml:space="preserve">Manufacturing-cluster PC1 loadings ~ Transformer 0.57, GOES 0.50, HV labor 0.60 (single dominant factor).</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Energization-Delay Simulation
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">95th-percentile energization delay when constraints are correlated vs assumed independent.</t>
-    </r>
+    <t xml:space="preserve">Manufacturing-cluster PC1 loadings ~ Transformer 0.54, GOES 0.57, HV labor 0.62 (single dominant factor).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energization-Delay Simulation
+95th-percentile energization delay when constraints are correlated vs assumed independent.</t>
   </si>
   <si>
     <t xml:space="preserve">Additive (sequential) stage-delay model; 300,000 draws; correlation from the manufacturing cluster. Computed in Python (numpy).</t>
@@ -373,49 +263,20 @@
     <t xml:space="preserve">p95 delay, correlated (months)</t>
   </si>
   <si>
-    <t xml:space="preserve">161.9</t>
-  </si>
-  <si>
     <t xml:space="preserve">p95 delay, independent (months)</t>
   </si>
   <si>
-    <t xml:space="preserve">157.8</t>
-  </si>
-  <si>
     <t xml:space="preserve">Understatement if assumed independent (years)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.34</t>
-  </si>
-  <si>
     <t xml:space="preserve">Paper's earlier claim (years)</t>
   </si>
   <si>
     <t xml:space="preserve">3.4 (not supported; corrected in the paper)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">GOES Demand Bridge
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9.5"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AI data centers' share of annual growth in grain-oriented electrical steel (GOES) demand.</t>
-    </r>
+    <t xml:space="preserve">GOES Demand Bridge
+AI data centers' share of annual growth in grain-oriented electrical steel (GOES) demand.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumption</t>
@@ -430,9 +291,6 @@
     <t xml:space="preserve">Global GOES consumption</t>
   </si>
   <si>
-    <t xml:space="preserve">2400</t>
-  </si>
-  <si>
     <t xml:space="preserve">kt/yr</t>
   </si>
   <si>
@@ -442,18 +300,12 @@
     <t xml:space="preserve">GOES demand growth (CAGR)</t>
   </si>
   <si>
-    <t xml:space="preserve">5.6%</t>
-  </si>
-  <si>
     <t xml:space="preserve">GOES market CAGR ~5-6%</t>
   </si>
   <si>
     <t xml:space="preserve">GOES per transformer</t>
   </si>
   <si>
-    <t xml:space="preserve">0.28</t>
-  </si>
-  <si>
     <t xml:space="preserve">t/MVA</t>
   </si>
   <si>
@@ -463,9 +315,6 @@
     <t xml:space="preserve">New AI data-center capacity, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">70</t>
-  </si>
-  <si>
     <t xml:space="preserve">GW</t>
   </si>
   <si>
@@ -473,9 +322,6 @@
   </si>
   <si>
     <t xml:space="preserve">Transformer MVA per MW IT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.5</t>
   </si>
   <si>
     <t xml:space="preserve">MVA/MW</t>
@@ -505,11 +351,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="165" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
-    <numFmt numFmtId="168" formatCode="#,##0"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="#,##0"/>
     <numFmt numFmtId="170" formatCode="0%"/>
   </numFmts>
   <fonts count="20">
@@ -746,7 +592,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -767,7 +613,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -779,7 +625,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -803,11 +649,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -815,15 +661,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -835,30 +677,38 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -867,23 +717,35 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1148,7 +1010,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="90"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1224,7 +1086,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="9" t="s">
         <v>16</v>
       </c>
@@ -1232,7 +1094,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="112.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
@@ -1289,7 +1151,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="15" t="s">
         <v>31</v>
       </c>
@@ -1317,14 +1179,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1339,516 +1199,521 @@
       <c r="G1" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H1" s="18"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="20" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>98</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B7" s="22" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>96</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>31</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>110</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>36</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>135</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B10" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>43</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>150</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>160</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F11" s="23" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>53</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>170</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+    </row>
+    <row r="14" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="23" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="C5" s="24" t="n">
-        <v>21</v>
-      </c>
-      <c r="D5" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="E5" s="23" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F5" s="24" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="23" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="C6" s="24" t="n">
-        <v>24</v>
-      </c>
-      <c r="D6" s="24" t="n">
-        <v>98</v>
-      </c>
-      <c r="E6" s="23" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F6" s="24" t="n">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="23" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="C7" s="24" t="n">
-        <v>27</v>
-      </c>
-      <c r="D7" s="24" t="n">
-        <v>96</v>
-      </c>
-      <c r="E7" s="23" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="F7" s="24" t="n">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" s="23" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="C8" s="24" t="n">
-        <v>31</v>
-      </c>
-      <c r="D8" s="24" t="n">
-        <v>110</v>
-      </c>
-      <c r="E8" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="24" t="n">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="C9" s="24" t="n">
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+    </row>
+    <row r="16" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="24" t="n">
-        <v>135</v>
-      </c>
-      <c r="E9" s="23" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F9" s="24" t="n">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="24" t="n">
-        <v>43</v>
-      </c>
-      <c r="D10" s="24" t="n">
-        <v>150</v>
-      </c>
-      <c r="E10" s="23" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="F10" s="24" t="n">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="23" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="C11" s="24" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" s="24" t="n">
-        <v>160</v>
-      </c>
-      <c r="E11" s="23" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="F11" s="24" t="n">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="23" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="C12" s="24" t="n">
-        <v>53</v>
-      </c>
-      <c r="D12" s="24" t="n">
-        <v>170</v>
-      </c>
-      <c r="E12" s="23" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="F12" s="24" t="n">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-    </row>
-    <row r="14" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-    </row>
-    <row r="16" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-    </row>
-    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="21" t="s">
+      <c r="D17" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="E17" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="20" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="26" t="n">
+      <c r="A18" s="21" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B18" s="25" t="n">
         <f aca="false">B6-B5</f>
         <v>0.2</v>
       </c>
-      <c r="C18" s="26" t="n">
+      <c r="C18" s="25" t="n">
         <f aca="false">C6-C5</f>
         <v>3</v>
       </c>
-      <c r="D18" s="26" t="n">
+      <c r="D18" s="25" t="n">
         <f aca="false">D6-D5</f>
         <v>-2</v>
       </c>
-      <c r="E18" s="26" t="n">
+      <c r="E18" s="25" t="n">
         <f aca="false">E6-E5</f>
         <v>-0.0999999999999996</v>
       </c>
-      <c r="F18" s="26" t="n">
+      <c r="F18" s="25" t="n">
         <f aca="false">F6-F5</f>
         <v>3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="26" t="n">
+      <c r="A19" s="21" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B19" s="25" t="n">
         <f aca="false">B7-B6</f>
         <v>0.2</v>
       </c>
-      <c r="C19" s="26" t="n">
+      <c r="C19" s="25" t="n">
         <f aca="false">C7-C6</f>
         <v>3</v>
       </c>
-      <c r="D19" s="26" t="n">
+      <c r="D19" s="25" t="n">
         <f aca="false">D7-D6</f>
         <v>-2</v>
       </c>
-      <c r="E19" s="26" t="n">
+      <c r="E19" s="25" t="n">
         <f aca="false">E7-E6</f>
         <v>-0.100000000000001</v>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F19" s="25" t="n">
         <f aca="false">F7-F6</f>
         <v>-2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="26" t="n">
+      <c r="A20" s="21" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B20" s="25" t="n">
         <f aca="false">B8-B7</f>
         <v>0.4</v>
       </c>
-      <c r="C20" s="26" t="n">
+      <c r="C20" s="25" t="n">
         <f aca="false">C8-C7</f>
         <v>4</v>
       </c>
-      <c r="D20" s="26" t="n">
+      <c r="D20" s="25" t="n">
         <f aca="false">D8-D7</f>
         <v>14</v>
       </c>
-      <c r="E20" s="26" t="n">
+      <c r="E20" s="25" t="n">
         <f aca="false">E8-E7</f>
         <v>-0.3</v>
       </c>
-      <c r="F20" s="26" t="n">
+      <c r="F20" s="25" t="n">
         <f aca="false">F8-F7</f>
         <v>7</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="26" t="n">
+      <c r="A21" s="21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B21" s="25" t="n">
         <f aca="false">B9-B8</f>
         <v>0.5</v>
       </c>
-      <c r="C21" s="26" t="n">
+      <c r="C21" s="25" t="n">
         <f aca="false">C9-C8</f>
         <v>5</v>
       </c>
-      <c r="D21" s="26" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">D9-D8</f>
         <v>25</v>
       </c>
-      <c r="E21" s="26" t="n">
+      <c r="E21" s="25" t="n">
         <f aca="false">E9-E8</f>
         <v>-0.1</v>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F21" s="25" t="n">
         <f aca="false">F9-F8</f>
         <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="26" t="n">
+      <c r="A22" s="21" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B22" s="25" t="n">
         <f aca="false">B10-B9</f>
         <v>0</v>
       </c>
-      <c r="C22" s="26" t="n">
+      <c r="C22" s="25" t="n">
         <f aca="false">C10-C9</f>
         <v>7</v>
       </c>
-      <c r="D22" s="26" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">D10-D9</f>
         <v>15</v>
       </c>
-      <c r="E22" s="26" t="n">
+      <c r="E22" s="25" t="n">
         <f aca="false">E10-E9</f>
         <v>-0.1</v>
       </c>
-      <c r="F22" s="26" t="n">
+      <c r="F22" s="25" t="n">
         <f aca="false">F10-F9</f>
         <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="26" t="n">
+      <c r="A23" s="21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B23" s="25" t="n">
         <f aca="false">B11-B10</f>
         <v>-0.4</v>
       </c>
-      <c r="C23" s="26" t="n">
+      <c r="C23" s="25" t="n">
         <f aca="false">C11-C10</f>
         <v>7</v>
       </c>
-      <c r="D23" s="26" t="n">
+      <c r="D23" s="25" t="n">
         <f aca="false">D11-D10</f>
         <v>10</v>
       </c>
-      <c r="E23" s="26" t="n">
+      <c r="E23" s="25" t="n">
         <f aca="false">E11-E10</f>
         <v>-0.0999999999999996</v>
       </c>
-      <c r="F23" s="26" t="n">
+      <c r="F23" s="25" t="n">
         <f aca="false">F11-F10</f>
         <v>10</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B24" s="26" t="n">
+      <c r="A24" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B24" s="25" t="n">
         <f aca="false">B12-B11</f>
         <v>0.2</v>
       </c>
-      <c r="C24" s="26" t="n">
+      <c r="C24" s="25" t="n">
         <f aca="false">C12-C11</f>
         <v>3</v>
       </c>
-      <c r="D24" s="26" t="n">
+      <c r="D24" s="25" t="n">
         <f aca="false">D12-D11</f>
         <v>10</v>
       </c>
-      <c r="E24" s="26" t="n">
+      <c r="E24" s="25" t="n">
         <f aca="false">E12-E11</f>
         <v>0</v>
       </c>
-      <c r="F24" s="26" t="n">
+      <c r="F24" s="25" t="n">
         <f aca="false">F12-F11</f>
         <v>7</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
     </row>
     <row r="26" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
     </row>
     <row r="27" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
+      <c r="A28" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
+      <c r="A29" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
     </row>
     <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
+      <c r="A30" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
     </row>
     <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
+      <c r="A31" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
     </row>
     <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="A32" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
     </row>
     <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
+      <c r="A33" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+    </row>
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="27" t="s">
+        <v>47</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1864,7 +1729,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.511811023622047" footer="0.511805555555556"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter>&amp;L&amp;"Arial,Regular"&amp;8 Simancas Capital | The Silicon-Power Gap&amp;R&amp;"Arial,Regular"&amp;8 &amp;A | Page &amp;P of &amp;N</oddFooter>
@@ -1881,16 +1746,14 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1903,199 +1766,199 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20"/>
-      <c r="B4" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="21" t="s">
-        <v>60</v>
+      <c r="A4" s="19"/>
+      <c r="B4" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="28" t="n">
+      <c r="A5" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!B18:B24,'Constraint Data'!B18:B24)</f>
         <v>1</v>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!B18:B24,'Constraint Data'!C18:C24)</f>
         <v>-0.604004174254959</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!B18:B24,'Constraint Data'!D18:D24)</f>
         <v>0.254043628982761</v>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E5" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!B18:B24,'Constraint Data'!E18:E24)</f>
         <v>-0.279426731036153</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!B18:B24,'Constraint Data'!F18:F24)</f>
         <v>-0.210674406485947</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="28" t="n">
+      <c r="A6" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!C18:C24,'Constraint Data'!B18:B24)</f>
         <v>-0.604004174254959</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!C18:C24,'Constraint Data'!C18:C24)</f>
         <v>1</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!C18:C24,'Constraint Data'!D18:D24)</f>
         <v>0.516711769954834</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!C18:C24,'Constraint Data'!E18:E24)</f>
         <v>-0.043796787185533</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!C18:C24,'Constraint Data'!F18:F24)</f>
         <v>0.740754632334416</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="29" t="n">
+      <c r="A7" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!D18:D24,'Constraint Data'!B18:B24)</f>
         <v>0.254043628982761</v>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!D18:D24,'Constraint Data'!C18:C24)</f>
         <v>0.516711769954834</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!D18:D24,'Constraint Data'!D18:D24)</f>
         <v>1</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!D18:D24,'Constraint Data'!E18:E24)</f>
         <v>-0.154221408822034</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!D18:D24,'Constraint Data'!F18:F24)</f>
         <v>0.831817573704798</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="29" t="n">
+      <c r="A8" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!E18:E24,'Constraint Data'!B18:B24)</f>
         <v>-0.279426731036153</v>
       </c>
-      <c r="C8" s="29" t="n">
+      <c r="C8" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!E18:E24,'Constraint Data'!C18:C24)</f>
         <v>-0.043796787185533</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!E18:E24,'Constraint Data'!D18:D24)</f>
         <v>-0.154221408822034</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!E18:E24,'Constraint Data'!E18:E24)</f>
         <v>1</v>
       </c>
-      <c r="F8" s="29" t="n">
+      <c r="F8" s="30" t="n">
         <f aca="false">CORREL('Constraint Data'!E18:E24,'Constraint Data'!F18:F24)</f>
         <v>-0.0235017788582069</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="28" t="n">
+      <c r="A9" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!F18:F24,'Constraint Data'!B18:B24)</f>
         <v>-0.210674406485947</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!F18:F24,'Constraint Data'!C18:C24)</f>
         <v>0.740754632334416</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!F18:F24,'Constraint Data'!D18:D24)</f>
         <v>0.831817573704798</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!F18:F24,'Constraint Data'!E18:E24)</f>
         <v>-0.0235017788582069</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="29" t="n">
         <f aca="false">CORREL('Constraint Data'!F18:F24,'Constraint Data'!F18:F24)</f>
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="27" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
+      <c r="A12" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
+      <c r="A13" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2127,13 +1990,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -2143,82 +2006,82 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="30"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="31"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="31"/>
+    </row>
+    <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="32" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="32" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="C7" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-    </row>
-    <row r="4" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="30"/>
-    </row>
-    <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B8" s="32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C8" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="20" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="31"/>
+    </row>
+    <row r="10" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="31"/>
+    </row>
+    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="30"/>
-    </row>
-    <row r="10" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="30"/>
-    </row>
-    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2249,13 +2112,13 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -2264,57 +2127,57 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="27"/>
+      <c r="A3" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="26"/>
     </row>
     <row r="4" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19"/>
-      <c r="B4" s="19"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>81</v>
+      <c r="A5" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>83</v>
+      <c r="A6" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="34" t="n">
+        <v>161.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>85</v>
+      <c r="A7" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="34" t="n">
+        <v>157.8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>87</v>
+      <c r="A8" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="35" t="n">
+        <v>0.34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>89</v>
+      <c r="A9" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2346,12 +2209,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -2359,222 +2222,222 @@
       <c r="E1" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="18"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="36" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="32" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="35" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>70</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="C4" s="21" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="B9" s="34" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C9" s="28" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="D9" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="32" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="25" t="n">
         <f aca="false">B5*B6</f>
         <v>134.4</v>
       </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="B12" s="26" t="n">
+      <c r="A12" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="25" t="n">
         <f aca="false">B8*1000*B9*B7/1000</f>
         <v>49</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="B13" s="33" t="n">
+      <c r="A13" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="37" t="n">
         <f aca="false">B12/B11</f>
         <v>0.364583333333333</v>
       </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
     </row>
     <row r="14" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
     </row>
     <row r="15" customFormat="false" ht="9" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
+      <c r="A16" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="B17" s="34" t="n">
+      <c r="A17" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="34" t="n">
+      <c r="C17" s="38" t="n">
         <v>2.5</v>
       </c>
-      <c r="D17" s="34" t="n">
+      <c r="D17" s="38" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="n">
+      <c r="A18" s="28" t="n">
         <v>50</v>
       </c>
-      <c r="B18" s="35" t="n">
+      <c r="B18" s="39" t="n">
         <f aca="false">50*1000*2*$B$7/1000/$B$11</f>
         <v>0.208333333333333</v>
       </c>
-      <c r="C18" s="35" t="n">
+      <c r="C18" s="39" t="n">
         <f aca="false">50*1000*2.5*$B$7/1000/$B$11</f>
         <v>0.260416666666667</v>
       </c>
-      <c r="D18" s="35" t="n">
+      <c r="D18" s="39" t="n">
         <f aca="false">50*1000*3*$B$7/1000/$B$11</f>
         <v>0.3125</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="n">
+      <c r="A19" s="28" t="n">
         <v>70</v>
       </c>
-      <c r="B19" s="35" t="n">
+      <c r="B19" s="39" t="n">
         <f aca="false">70*1000*2*$B$7/1000/$B$11</f>
         <v>0.291666666666667</v>
       </c>
-      <c r="C19" s="35" t="n">
+      <c r="C19" s="39" t="n">
         <f aca="false">70*1000*2.5*$B$7/1000/$B$11</f>
         <v>0.364583333333333</v>
       </c>
-      <c r="D19" s="35" t="n">
+      <c r="D19" s="39" t="n">
         <f aca="false">70*1000*3*$B$7/1000/$B$11</f>
         <v>0.4375</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="n">
+      <c r="A20" s="28" t="n">
         <v>90</v>
       </c>
-      <c r="B20" s="35" t="n">
+      <c r="B20" s="39" t="n">
         <f aca="false">90*1000*2*$B$7/1000/$B$11</f>
         <v>0.375</v>
       </c>
-      <c r="C20" s="35" t="n">
+      <c r="C20" s="39" t="n">
         <f aca="false">90*1000*2.5*$B$7/1000/$B$11</f>
         <v>0.46875</v>
       </c>
-      <c r="D20" s="35" t="n">
+      <c r="D20" s="39" t="n">
         <f aca="false">90*1000*3*$B$7/1000/$B$11</f>
         <v>0.5625</v>
       </c>

</xml_diff>